<commit_message>
updated inventory for Uganda (broke out pasture paddock range, which doesn't appear to be part of their inventory, though the NC3 says is a signifiacnt source of N2O emissions (table 2.59)
</commit_message>
<xml_diff>
--- a/data_processing/input_data/historical_inventory_comparison_clews_sisepuede_2019.xlsx
+++ b/data_processing/input_data/historical_inventory_comparison_clews_sisepuede_2019.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/ssp_uganda_data/data_processing/input_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F6364C-3D0A-2F4E-B1CB-E4F042ADC4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C970B5B6-8E77-AE44-9BE1-6D44C85A11B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2720" yWindow="500" windowWidth="31060" windowHeight="18100" xr2:uid="{67B887B1-FF49-CC44-8025-2B1602161908}"/>
+    <workbookView xWindow="8540" yWindow="1540" windowWidth="31060" windowHeight="18100" xr2:uid="{67B887B1-FF49-CC44-8025-2B1602161908}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -646,28 +646,28 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -1020,10 +1020,10 @@
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="53"/>
+      <c r="E1" s="51"/>
       <c r="F1" s="4"/>
       <c r="G1" s="5"/>
     </row>
@@ -1050,10 +1050,10 @@
       <c r="A3" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="B3" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="49"/>
+      <c r="C3" s="48"/>
       <c r="D3" s="14">
         <v>0</v>
       </c>
@@ -1067,10 +1067,10 @@
       <c r="A4" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="54"/>
+      <c r="C4" s="52"/>
       <c r="D4" s="21">
         <v>1.36</v>
       </c>
@@ -1086,10 +1086,10 @@
       <c r="A5" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="49" t="s">
+      <c r="B5" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="49"/>
+      <c r="C5" s="48"/>
       <c r="D5" s="26">
         <v>4.2</v>
       </c>
@@ -1105,10 +1105,10 @@
       <c r="A6" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="54" t="s">
+      <c r="B6" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="54"/>
+      <c r="C6" s="52"/>
       <c r="D6" s="21">
         <v>3.1</v>
       </c>
@@ -1124,10 +1124,10 @@
       <c r="A7" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="49"/>
+      <c r="C7" s="48"/>
       <c r="D7" s="26">
         <v>2.97</v>
       </c>
@@ -1143,10 +1143,10 @@
       <c r="A8" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="54" t="s">
+      <c r="B8" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="54"/>
+      <c r="C8" s="52"/>
       <c r="D8" s="21">
         <v>0.36</v>
       </c>
@@ -1162,10 +1162,10 @@
       <c r="A9" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="49" t="s">
+      <c r="B9" s="48" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="49"/>
+      <c r="C9" s="48"/>
       <c r="D9" s="26">
         <v>27.3</v>
       </c>
@@ -1221,7 +1221,7 @@
       <c r="C12" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="50" t="s">
+      <c r="D12" s="47" t="s">
         <v>33</v>
       </c>
       <c r="E12" s="31">
@@ -1239,7 +1239,7 @@
       <c r="C13" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="50"/>
+      <c r="D13" s="47"/>
       <c r="E13" s="31">
         <v>5.4600000000000004E-4</v>
       </c>
@@ -1255,7 +1255,7 @@
       <c r="C14" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="50"/>
+      <c r="D14" s="47"/>
       <c r="E14" s="31">
         <v>7.0433999999999997E-2</v>
       </c>
@@ -1271,7 +1271,7 @@
       <c r="C15" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="50"/>
+      <c r="D15" s="47"/>
       <c r="E15" s="31">
         <v>0</v>
       </c>
@@ -1287,7 +1287,7 @@
       <c r="C16" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="50"/>
+      <c r="D16" s="47"/>
       <c r="E16" s="33">
         <v>4.5830000000000003E-3</v>
       </c>
@@ -1303,7 +1303,7 @@
       <c r="C17" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="50"/>
+      <c r="D17" s="47"/>
       <c r="E17" s="33">
         <v>1.123E-2</v>
       </c>
@@ -1319,7 +1319,7 @@
       <c r="C18" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="50"/>
+      <c r="D18" s="47"/>
       <c r="E18" s="31">
         <v>0.23899999999999999</v>
       </c>
@@ -1335,7 +1335,7 @@
       <c r="C19" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="50"/>
+      <c r="D19" s="47"/>
       <c r="E19" s="31">
         <v>0.40160000000000001</v>
       </c>
@@ -1351,7 +1351,7 @@
       <c r="C20" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="50"/>
+      <c r="D20" s="47"/>
       <c r="E20" s="31">
         <v>1.4790000000000001</v>
       </c>
@@ -1364,10 +1364,10 @@
       <c r="A21" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="49" t="s">
+      <c r="B21" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="49"/>
+      <c r="C21" s="48"/>
       <c r="D21" s="26">
         <f>+D22+D24</f>
         <v>55.699999999999996</v>
@@ -1388,7 +1388,7 @@
       <c r="C22" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="D22" s="51">
+      <c r="D22" s="49">
         <v>65.099999999999994</v>
       </c>
       <c r="E22" s="31">
@@ -1405,7 +1405,7 @@
       <c r="C23" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="51"/>
+      <c r="D23" s="49"/>
       <c r="E23" s="31">
         <v>13.3</v>
       </c>
@@ -1432,10 +1432,10 @@
       <c r="A25" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="49" t="s">
+      <c r="B25" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="C25" s="49"/>
+      <c r="C25" s="48"/>
       <c r="D25" s="26">
         <v>7.84</v>
       </c>
@@ -1451,10 +1451,10 @@
       <c r="A26" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="54" t="s">
+      <c r="B26" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="C26" s="54"/>
+      <c r="C26" s="52"/>
       <c r="D26" s="21">
         <v>5.7</v>
       </c>
@@ -1472,11 +1472,11 @@
       <c r="E27" s="36"/>
     </row>
     <row r="28" spans="1:7" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="48" t="s">
+      <c r="A28" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
+      <c r="B28" s="54"/>
+      <c r="C28" s="54"/>
       <c r="D28" s="38"/>
       <c r="E28" s="39"/>
       <c r="F28" s="40" t="s">
@@ -1488,10 +1488,10 @@
       <c r="A29" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="B29" s="47" t="s">
+      <c r="B29" s="53" t="s">
         <v>19</v>
       </c>
-      <c r="C29" s="47"/>
+      <c r="C29" s="53"/>
       <c r="D29" s="30"/>
       <c r="E29" s="31" t="s">
         <v>22</v>
@@ -1504,10 +1504,10 @@
       <c r="A30" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="47" t="s">
+      <c r="B30" s="53" t="s">
         <v>45</v>
       </c>
-      <c r="C30" s="47"/>
+      <c r="C30" s="53"/>
       <c r="D30" s="30"/>
       <c r="E30" s="31" t="s">
         <v>22</v>
@@ -1520,10 +1520,10 @@
       <c r="A31" s="44" t="s">
         <v>39</v>
       </c>
-      <c r="B31" s="47" t="s">
+      <c r="B31" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="47"/>
+      <c r="C31" s="53"/>
       <c r="D31" s="45" t="s">
         <v>22</v>
       </c>
@@ -1553,6 +1553,13 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
     <mergeCell ref="D12:D20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B9:C9"/>
@@ -1563,13 +1570,6 @@
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>